<commit_message>
Make the Research Hub demo a hypothetical weighted portfolio
Add explicit weights totaling 100%, compare equal weights and company counts, and preserve the selected basis in saved copies and reports. Keep captured SEC facts unchanged and align all downloadable templates.
</commit_message>
<xml_diff>
--- a/public/portfolio/portfolio-demo-100.xlsx
+++ b/public/portfolio/portfolio-demo-100.xlsx
@@ -120,6 +120,9 @@
           <t xml:space="preserve">AAPL</t>
         </is>
       </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -127,6 +130,9 @@
           <t xml:space="preserve">MSFT</t>
         </is>
       </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -134,6 +140,9 @@
           <t xml:space="preserve">NVDA</t>
         </is>
       </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -141,6 +150,9 @@
           <t xml:space="preserve">ORCL</t>
         </is>
       </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -148,6 +160,9 @@
           <t xml:space="preserve">ADBE</t>
         </is>
       </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -155,6 +170,9 @@
           <t xml:space="preserve">CRM</t>
         </is>
       </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -162,6 +180,9 @@
           <t xml:space="preserve">AMD</t>
         </is>
       </c>
+      <c r="E8">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -169,6 +190,9 @@
           <t xml:space="preserve">INTC</t>
         </is>
       </c>
+      <c r="E9">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -176,6 +200,9 @@
           <t xml:space="preserve">CSCO</t>
         </is>
       </c>
+      <c r="E10">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -183,6 +210,9 @@
           <t xml:space="preserve">IBM</t>
         </is>
       </c>
+      <c r="E11">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -190,6 +220,9 @@
           <t xml:space="preserve">AMZN</t>
         </is>
       </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -197,6 +230,9 @@
           <t xml:space="preserve">TSLA</t>
         </is>
       </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -204,6 +240,9 @@
           <t xml:space="preserve">HD</t>
         </is>
       </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -211,6 +250,9 @@
           <t xml:space="preserve">LOW</t>
         </is>
       </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -218,6 +260,9 @@
           <t xml:space="preserve">NKE</t>
         </is>
       </c>
+      <c r="E16">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -225,6 +270,9 @@
           <t xml:space="preserve">MCD</t>
         </is>
       </c>
+      <c r="E17">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -232,6 +280,9 @@
           <t xml:space="preserve">SBUX</t>
         </is>
       </c>
+      <c r="E18">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -239,6 +290,9 @@
           <t xml:space="preserve">TGT</t>
         </is>
       </c>
+      <c r="E19">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -246,6 +300,9 @@
           <t xml:space="preserve">TJX</t>
         </is>
       </c>
+      <c r="E20">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -253,6 +310,9 @@
           <t xml:space="preserve">BKNG</t>
         </is>
       </c>
+      <c r="E21">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -260,6 +320,9 @@
           <t xml:space="preserve">WMT</t>
         </is>
       </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -267,6 +330,9 @@
           <t xml:space="preserve">COST</t>
         </is>
       </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -274,6 +340,9 @@
           <t xml:space="preserve">PG</t>
         </is>
       </c>
+      <c r="E24">
+        <v>2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -281,6 +350,9 @@
           <t xml:space="preserve">KO</t>
         </is>
       </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -288,6 +360,9 @@
           <t xml:space="preserve">PEP</t>
         </is>
       </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -295,6 +370,9 @@
           <t xml:space="preserve">MDLZ</t>
         </is>
       </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -302,6 +380,9 @@
           <t xml:space="preserve">CL</t>
         </is>
       </c>
+      <c r="E28">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -309,6 +390,9 @@
           <t xml:space="preserve">KMB</t>
         </is>
       </c>
+      <c r="E29">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -316,6 +400,9 @@
           <t xml:space="preserve">GIS</t>
         </is>
       </c>
+      <c r="E30">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -323,6 +410,9 @@
           <t xml:space="preserve">KHC</t>
         </is>
       </c>
+      <c r="E31">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -330,6 +420,9 @@
           <t xml:space="preserve">JPM</t>
         </is>
       </c>
+      <c r="E32">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -337,6 +430,9 @@
           <t xml:space="preserve">BAC</t>
         </is>
       </c>
+      <c r="E33">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -344,6 +440,9 @@
           <t xml:space="preserve">WFC</t>
         </is>
       </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -351,6 +450,9 @@
           <t xml:space="preserve">C</t>
         </is>
       </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -358,6 +460,9 @@
           <t xml:space="preserve">GS</t>
         </is>
       </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -365,6 +470,9 @@
           <t xml:space="preserve">MS</t>
         </is>
       </c>
+      <c r="E37">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -372,6 +480,9 @@
           <t xml:space="preserve">AXP</t>
         </is>
       </c>
+      <c r="E38">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -379,6 +490,9 @@
           <t xml:space="preserve">SCHW</t>
         </is>
       </c>
+      <c r="E39">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -386,6 +500,9 @@
           <t xml:space="preserve">USB</t>
         </is>
       </c>
+      <c r="E40">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -393,6 +510,9 @@
           <t xml:space="preserve">PNC</t>
         </is>
       </c>
+      <c r="E41">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -400,6 +520,9 @@
           <t xml:space="preserve">UNH</t>
         </is>
       </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -407,6 +530,9 @@
           <t xml:space="preserve">JNJ</t>
         </is>
       </c>
+      <c r="E43">
+        <v>5</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -414,6 +540,9 @@
           <t xml:space="preserve">LLY</t>
         </is>
       </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -421,6 +550,9 @@
           <t xml:space="preserve">MRK</t>
         </is>
       </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -428,6 +560,9 @@
           <t xml:space="preserve">ABBV</t>
         </is>
       </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -435,6 +570,9 @@
           <t xml:space="preserve">ABT</t>
         </is>
       </c>
+      <c r="E47">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -442,6 +580,9 @@
           <t xml:space="preserve">TMO</t>
         </is>
       </c>
+      <c r="E48">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -449,6 +590,9 @@
           <t xml:space="preserve">DHR</t>
         </is>
       </c>
+      <c r="E49">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -456,6 +600,9 @@
           <t xml:space="preserve">AMGN</t>
         </is>
       </c>
+      <c r="E50">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -463,6 +610,9 @@
           <t xml:space="preserve">GILD</t>
         </is>
       </c>
+      <c r="E51">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -470,6 +620,9 @@
           <t xml:space="preserve">CAT</t>
         </is>
       </c>
+      <c r="E52">
+        <v>2</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -477,6 +630,9 @@
           <t xml:space="preserve">DE</t>
         </is>
       </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -484,6 +640,9 @@
           <t xml:space="preserve">GE</t>
         </is>
       </c>
+      <c r="E54">
+        <v>2</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -491,6 +650,9 @@
           <t xml:space="preserve">HON</t>
         </is>
       </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -498,6 +660,9 @@
           <t xml:space="preserve">UPS</t>
         </is>
       </c>
+      <c r="E56">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -505,6 +670,9 @@
           <t xml:space="preserve">FDX</t>
         </is>
       </c>
+      <c r="E57">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -512,6 +680,9 @@
           <t xml:space="preserve">RTX</t>
         </is>
       </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -519,6 +690,9 @@
           <t xml:space="preserve">LMT</t>
         </is>
       </c>
+      <c r="E59">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -526,6 +700,9 @@
           <t xml:space="preserve">NOC</t>
         </is>
       </c>
+      <c r="E60">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -533,6 +710,9 @@
           <t xml:space="preserve">GD</t>
         </is>
       </c>
+      <c r="E61">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -540,6 +720,9 @@
           <t xml:space="preserve">XOM</t>
         </is>
       </c>
+      <c r="E62">
+        <v>5</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -547,6 +730,9 @@
           <t xml:space="preserve">CVX</t>
         </is>
       </c>
+      <c r="E63">
+        <v>2</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -554,6 +740,9 @@
           <t xml:space="preserve">COP</t>
         </is>
       </c>
+      <c r="E64">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -561,6 +750,9 @@
           <t xml:space="preserve">EOG</t>
         </is>
       </c>
+      <c r="E65">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -568,6 +760,9 @@
           <t xml:space="preserve">SLB</t>
         </is>
       </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -575,6 +770,9 @@
           <t xml:space="preserve">OXY</t>
         </is>
       </c>
+      <c r="E67">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -582,6 +780,9 @@
           <t xml:space="preserve">PSX</t>
         </is>
       </c>
+      <c r="E68">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -589,6 +790,9 @@
           <t xml:space="preserve">VLO</t>
         </is>
       </c>
+      <c r="E69">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -596,6 +800,9 @@
           <t xml:space="preserve">MPC</t>
         </is>
       </c>
+      <c r="E70">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -603,6 +810,9 @@
           <t xml:space="preserve">KMI</t>
         </is>
       </c>
+      <c r="E71">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -610,6 +820,9 @@
           <t xml:space="preserve">NEE</t>
         </is>
       </c>
+      <c r="E72">
+        <v>2</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -617,6 +830,9 @@
           <t xml:space="preserve">DUK</t>
         </is>
       </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -624,6 +840,9 @@
           <t xml:space="preserve">SO</t>
         </is>
       </c>
+      <c r="E74">
+        <v>1</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -631,6 +850,9 @@
           <t xml:space="preserve">AEP</t>
         </is>
       </c>
+      <c r="E75">
+        <v>1</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -638,6 +860,9 @@
           <t xml:space="preserve">EXC</t>
         </is>
       </c>
+      <c r="E76">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -645,6 +870,9 @@
           <t xml:space="preserve">SRE</t>
         </is>
       </c>
+      <c r="E77">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -652,6 +880,9 @@
           <t xml:space="preserve">XEL</t>
         </is>
       </c>
+      <c r="E78">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -659,6 +890,9 @@
           <t xml:space="preserve">WEC</t>
         </is>
       </c>
+      <c r="E79">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -666,6 +900,9 @@
           <t xml:space="preserve">ED</t>
         </is>
       </c>
+      <c r="E80">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -673,6 +910,9 @@
           <t xml:space="preserve">D</t>
         </is>
       </c>
+      <c r="E81">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -680,6 +920,9 @@
           <t xml:space="preserve">GOOGL</t>
         </is>
       </c>
+      <c r="E82">
+        <v>2</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -687,6 +930,9 @@
           <t xml:space="preserve">META</t>
         </is>
       </c>
+      <c r="E83">
+        <v>2</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -694,6 +940,9 @@
           <t xml:space="preserve">NFLX</t>
         </is>
       </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -701,6 +950,9 @@
           <t xml:space="preserve">DIS</t>
         </is>
       </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -708,6 +960,9 @@
           <t xml:space="preserve">CMCSA</t>
         </is>
       </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -715,6 +970,9 @@
           <t xml:space="preserve">VZ</t>
         </is>
       </c>
+      <c r="E87">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -722,6 +980,9 @@
           <t xml:space="preserve">T</t>
         </is>
       </c>
+      <c r="E88">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -729,6 +990,9 @@
           <t xml:space="preserve">CHTR</t>
         </is>
       </c>
+      <c r="E89">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -736,6 +1000,9 @@
           <t xml:space="preserve">TTWO</t>
         </is>
       </c>
+      <c r="E90">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -743,6 +1010,9 @@
           <t xml:space="preserve">WBD</t>
         </is>
       </c>
+      <c r="E91">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -750,6 +1020,9 @@
           <t xml:space="preserve">LIN</t>
         </is>
       </c>
+      <c r="E92">
+        <v>2</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -757,6 +1030,9 @@
           <t xml:space="preserve">APD</t>
         </is>
       </c>
+      <c r="E93">
+        <v>1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -764,6 +1040,9 @@
           <t xml:space="preserve">SHW</t>
         </is>
       </c>
+      <c r="E94">
+        <v>1</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -771,6 +1050,9 @@
           <t xml:space="preserve">FCX</t>
         </is>
       </c>
+      <c r="E95">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -778,6 +1060,9 @@
           <t xml:space="preserve">NEM</t>
         </is>
       </c>
+      <c r="E96">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -785,6 +1070,9 @@
           <t xml:space="preserve">NUE</t>
         </is>
       </c>
+      <c r="E97">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -792,6 +1080,9 @@
           <t xml:space="preserve">PLD</t>
         </is>
       </c>
+      <c r="E98">
+        <v>2</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -799,6 +1090,9 @@
           <t xml:space="preserve">AMT</t>
         </is>
       </c>
+      <c r="E99">
+        <v>1</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -806,12 +1100,18 @@
           <t xml:space="preserve">SPG</t>
         </is>
       </c>
+      <c r="E100">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
           <t xml:space="preserve">O</t>
         </is>
+      </c>
+      <c r="E101">
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>
@@ -827,7 +1127,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">100-company research demo</t>
+          <t xml:space="preserve">Hypothetical weighted portfolio · 100-company demo</t>
         </is>
       </c>
     </row>
@@ -839,7 +1139,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Upload this workbook in Research Hub → Portfolio research. The Holdings sheet is prefilled with exactly 100 company tickers.</t>
+          <t xml:space="preserve">Upload this workbook in Research Hub → Portfolio research. The Holdings sheet contains 100 company tickers and hypothetical weight_pct values totaling 100%. Select Weighted portfolio — supplied weight_pct in Allocation settings after import.</t>
         </is>
       </c>
     </row>
@@ -851,7 +1151,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review company financial metrics, reporting periods, SEC filing sources, coverage and industry groups. Open the captured example at https://secedgarterminal.com/workspace/demo.</t>
+          <t xml:space="preserve">Explore weighted issuer and industry concentration, evidence coverage, scenarios, company metrics and SEC filing sources. Open https://secedgarterminal.com/workspace/demo to compare the example with equal weights or company counts.</t>
         </is>
       </c>
     </row>
@@ -870,46 +1170,58 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Optional fields</t>
+          <t xml:space="preserve">Hypothetical weights</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ticker-only input is sufficient. Weights, market values, shares and private notes are intentionally blank. No equal-weight allocation is assumed.</t>
+          <t xml:space="preserve">Fixed hypothetical weights: 5 companies at 5% each, 15 at 2%, 30 at 1%, and 50 at 0.3%, totaling 100%. These educational inputs are not derived from market prices, company fundamentals, an index, or actual holdings and are not investment recommendations.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dates</t>
+          <t xml:space="preserve">Weight units</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The example analysis is a dated capture. Running research retrieves current available public evidence; results and coverage may differ.</t>
+          <t xml:space="preserve">weight_pct uses percentage points: 5 means 5%, and 0.3 means 0.3%. These are literal values. The remaining input fields are blank. Clear the weights to use your own company research list.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limits</t>
+          <t xml:space="preserve">Dates</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">The import supports at most 100 rows. Replace existing tickers before adding more. Cells contain literal values, with no formulas or macros.</t>
+          <t xml:space="preserve">The example analysis is a dated capture. Running research retrieves current available public evidence; results and coverage may differ.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Limits</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The import supports at most 100 rows. Replace existing tickers before adding more. Cells contain literal values, with no formulas or macros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Privacy</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t xml:space="preserve">Imported notes remain in your browser. Interactive research sends company identifiers, not private allocations or notes.</t>
         </is>

</xml_diff>